<commit_message>
Dashboard i18n — step 9: cotización detail subcomponents (timeline, line-items-editor, firma-panel)
- line-items-editor: full es/en strings + currency-aware amounts via moneda/locale
- firma-panel: full es/en strings, locale-aware signed date
- timeline already lang-aware; wired lang/locale from detail page
- DETAIL_STRINGS extended with lineItemsEditor + firmaPanel namespaces

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dealforge-urls.xlsx
+++ b/dealforge-urls.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Nexus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4342C6D0-3159-4687-BF11-D3CD3C516631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE3E0FA-BF7C-4BC8-8B18-321164A958A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16354" yWindow="-103" windowWidth="16663" windowHeight="8743" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,25 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">URLs!$A$1:$C$59</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="73">
   <si>
     <t>URL</t>
   </si>
@@ -224,13 +237,31 @@
   </si>
   <si>
     <t>Requested</t>
+  </si>
+  <si>
+    <t>https://dealforge.es/calculadora-roi</t>
+  </si>
+  <si>
+    <t>https://dealforge.es/comparar</t>
+  </si>
+  <si>
+    <t>https://dealforge.es/comparar/dealforge-vs-holded</t>
+  </si>
+  <si>
+    <t>https://dealforge.es/comparar/dealforge-vs-hubspot</t>
+  </si>
+  <si>
+    <t>https://dealforge.es/comparar/dealforge-vs-excel</t>
+  </si>
+  <si>
+    <t>https://dealforge.es/glosario</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -252,6 +283,14 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -322,10 +361,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -349,8 +389,10 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -653,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="75" customWidth="1"/>
@@ -954,8 +996,8 @@
       <c r="B27" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>5</v>
+      <c r="C27" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
@@ -965,8 +1007,8 @@
       <c r="B28" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="4" t="s">
-        <v>5</v>
+      <c r="C28" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
@@ -976,8 +1018,8 @@
       <c r="B29" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>5</v>
+      <c r="C29" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
@@ -987,8 +1029,8 @@
       <c r="B30" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>5</v>
+      <c r="C30" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
@@ -998,8 +1040,8 @@
       <c r="B31" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>5</v>
+      <c r="C31" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
@@ -1009,8 +1051,8 @@
       <c r="B32" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C32" s="4" t="s">
-        <v>5</v>
+      <c r="C32" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
@@ -1020,8 +1062,8 @@
       <c r="B33" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C33" s="4" t="s">
-        <v>5</v>
+      <c r="C33" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
@@ -1031,8 +1073,8 @@
       <c r="B34" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C34" s="4" t="s">
-        <v>5</v>
+      <c r="C34" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
@@ -1042,8 +1084,8 @@
       <c r="B35" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C35" s="4" t="s">
-        <v>5</v>
+      <c r="C35" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
@@ -1053,8 +1095,8 @@
       <c r="B36" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C36" s="4" t="s">
-        <v>5</v>
+      <c r="C36" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
@@ -1064,8 +1106,8 @@
       <c r="B37" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="4" t="s">
-        <v>5</v>
+      <c r="C37" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
@@ -1075,8 +1117,8 @@
       <c r="B38" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C38" s="4" t="s">
-        <v>5</v>
+      <c r="C38" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
@@ -1086,8 +1128,8 @@
       <c r="B39" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C39" s="4" t="s">
-        <v>5</v>
+      <c r="C39" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
@@ -1097,8 +1139,8 @@
       <c r="B40" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C40" s="4" t="s">
-        <v>5</v>
+      <c r="C40" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
@@ -1108,8 +1150,8 @@
       <c r="B41" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C41" s="4" t="s">
-        <v>5</v>
+      <c r="C41" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
@@ -1119,8 +1161,8 @@
       <c r="B42" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C42" s="4" t="s">
-        <v>5</v>
+      <c r="C42" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
@@ -1130,8 +1172,8 @@
       <c r="B43" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C43" s="4" t="s">
-        <v>5</v>
+      <c r="C43" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
@@ -1141,8 +1183,8 @@
       <c r="B44" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C44" s="4" t="s">
-        <v>5</v>
+      <c r="C44" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
@@ -1152,8 +1194,8 @@
       <c r="B45" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C45" s="4" t="s">
-        <v>5</v>
+      <c r="C45" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
@@ -1163,8 +1205,8 @@
       <c r="B46" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C46" s="4" t="s">
-        <v>5</v>
+      <c r="C46" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
@@ -1174,8 +1216,8 @@
       <c r="B47" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C47" s="4" t="s">
-        <v>5</v>
+      <c r="C47" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
@@ -1185,8 +1227,8 @@
       <c r="B48" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C48" s="4" t="s">
-        <v>5</v>
+      <c r="C48" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
@@ -1196,8 +1238,8 @@
       <c r="B49" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C49" s="4" t="s">
-        <v>5</v>
+      <c r="C49" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
@@ -1207,8 +1249,8 @@
       <c r="B50" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C50" s="4" t="s">
-        <v>5</v>
+      <c r="C50" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
@@ -1218,8 +1260,8 @@
       <c r="B51" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C51" s="4" t="s">
-        <v>5</v>
+      <c r="C51" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
@@ -1229,8 +1271,8 @@
       <c r="B52" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C52" s="4" t="s">
-        <v>5</v>
+      <c r="C52" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
@@ -1240,8 +1282,8 @@
       <c r="B53" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C53" s="4" t="s">
-        <v>5</v>
+      <c r="C53" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
@@ -1251,8 +1293,8 @@
       <c r="B54" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C54" s="4" t="s">
-        <v>5</v>
+      <c r="C54" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
@@ -1262,8 +1304,8 @@
       <c r="B55" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C55" s="4" t="s">
-        <v>5</v>
+      <c r="C55" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
@@ -1273,8 +1315,8 @@
       <c r="B56" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C56" s="4" t="s">
-        <v>5</v>
+      <c r="C56" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
@@ -1284,8 +1326,8 @@
       <c r="B57" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C57" s="4" t="s">
-        <v>5</v>
+      <c r="C57" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
@@ -1295,8 +1337,8 @@
       <c r="B58" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C58" s="4" t="s">
-        <v>5</v>
+      <c r="C58" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
@@ -1306,12 +1348,81 @@
       <c r="B59" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C59" s="4" t="s">
-        <v>5</v>
+      <c r="C59" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>69</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>70</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C63" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>71</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>72</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C65" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:C59" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <hyperlinks>
+    <hyperlink ref="A61" r:id="rId1" xr:uid="{AF0DF64A-6F78-4E35-9CC2-2233A2DD9C73}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>